<commit_message>
updated strategy templates and some transformations
</commit_message>
<xml_diff>
--- a/data_processing/transformations/templates/calibrated/uganda/model_input_variables_uganda_ce_calibrated.xlsx
+++ b/data_processing/transformations/templates/calibrated/uganda/model_input_variables_uganda_ce_calibrated.xlsx
@@ -43213,133 +43213,133 @@
         <v>0</v>
       </c>
       <c r="W4">
+        <v>0.002325581395348837</v>
+      </c>
+      <c r="X4">
+        <v>0.004651162790697674</v>
+      </c>
+      <c r="Y4">
         <v>0.006976744186046512</v>
       </c>
-      <c r="X4">
+      <c r="Z4">
+        <v>0.009302325581395349</v>
+      </c>
+      <c r="AA4">
+        <v>0.01162790697674419</v>
+      </c>
+      <c r="AB4">
         <v>0.01395348837209302</v>
       </c>
-      <c r="Y4">
-        <v>0.02093023255813953</v>
-      </c>
-      <c r="Z4">
+      <c r="AC4">
+        <v>0.01627906976744186</v>
+      </c>
+      <c r="AD4">
+        <v>0.0186046511627907</v>
+      </c>
+      <c r="AE4">
+        <v>0.02093023255813954</v>
+      </c>
+      <c r="AF4">
+        <v>0.02325581395348837</v>
+      </c>
+      <c r="AG4">
+        <v>0.02558139534883721</v>
+      </c>
+      <c r="AH4">
         <v>0.02790697674418605</v>
       </c>
-      <c r="AA4">
+      <c r="AI4">
+        <v>0.03023255813953488</v>
+      </c>
+      <c r="AJ4">
+        <v>0.03255813953488373</v>
+      </c>
+      <c r="AK4">
         <v>0.03488372093023256</v>
       </c>
-      <c r="AB4">
-        <v>0.04186046511627907</v>
-      </c>
-      <c r="AC4">
+      <c r="AL4">
+        <v>0.03720930232558139</v>
+      </c>
+      <c r="AM4">
+        <v>0.03953488372093023</v>
+      </c>
+      <c r="AN4">
+        <v>0.04186046511627908</v>
+      </c>
+      <c r="AO4">
+        <v>0.04418604651162791</v>
+      </c>
+      <c r="AP4">
+        <v>0.04651162790697674</v>
+      </c>
+      <c r="AQ4">
         <v>0.04883720930232558</v>
       </c>
-      <c r="AD4">
+      <c r="AR4">
+        <v>0.05116279069767442</v>
+      </c>
+      <c r="AS4">
+        <v>0.05348837209302326</v>
+      </c>
+      <c r="AT4">
         <v>0.05581395348837209</v>
       </c>
-      <c r="AE4">
+      <c r="AU4">
+        <v>0.05813953488372094</v>
+      </c>
+      <c r="AV4">
+        <v>0.06046511627906977</v>
+      </c>
+      <c r="AW4">
         <v>0.06279069767441861</v>
       </c>
-      <c r="AF4">
+      <c r="AX4">
+        <v>0.06511627906976745</v>
+      </c>
+      <c r="AY4">
+        <v>0.06744186046511629</v>
+      </c>
+      <c r="AZ4">
         <v>0.06976744186046512</v>
       </c>
-      <c r="AG4">
+      <c r="BA4">
+        <v>0.07209302325581395</v>
+      </c>
+      <c r="BB4">
+        <v>0.07441860465116279</v>
+      </c>
+      <c r="BC4">
         <v>0.07674418604651163</v>
       </c>
-      <c r="AH4">
-        <v>0.08372093023255814</v>
-      </c>
-      <c r="AI4">
-        <v>0.09069767441860464</v>
-      </c>
-      <c r="AJ4">
+      <c r="BD4">
+        <v>0.07906976744186046</v>
+      </c>
+      <c r="BE4">
+        <v>0.08139534883720931</v>
+      </c>
+      <c r="BF4">
+        <v>0.08372093023255815</v>
+      </c>
+      <c r="BG4">
+        <v>0.08604651162790698</v>
+      </c>
+      <c r="BH4">
+        <v>0.08837209302325583</v>
+      </c>
+      <c r="BI4">
+        <v>0.09069767441860466</v>
+      </c>
+      <c r="BJ4">
+        <v>0.09302325581395349</v>
+      </c>
+      <c r="BK4">
+        <v>0.09534883720930233</v>
+      </c>
+      <c r="BL4">
         <v>0.09767441860465116</v>
       </c>
-      <c r="AK4">
-        <v>0.1046511627906977</v>
-      </c>
-      <c r="AL4">
-        <v>0.1116279069767442</v>
-      </c>
-      <c r="AM4">
-        <v>0.1186046511627907</v>
-      </c>
-      <c r="AN4">
-        <v>0.1255813953488372</v>
-      </c>
-      <c r="AO4">
-        <v>0.1325581395348837</v>
-      </c>
-      <c r="AP4">
-        <v>0.1395348837209302</v>
-      </c>
-      <c r="AQ4">
-        <v>0.1465116279069767</v>
-      </c>
-      <c r="AR4">
-        <v>0.1534883720930233</v>
-      </c>
-      <c r="AS4">
-        <v>0.1604651162790698</v>
-      </c>
-      <c r="AT4">
-        <v>0.1674418604651163</v>
-      </c>
-      <c r="AU4">
-        <v>0.1744186046511628</v>
-      </c>
-      <c r="AV4">
-        <v>0.1813953488372093</v>
-      </c>
-      <c r="AW4">
-        <v>0.1883720930232558</v>
-      </c>
-      <c r="AX4">
-        <v>0.1953488372093023</v>
-      </c>
-      <c r="AY4">
-        <v>0.2023255813953488</v>
-      </c>
-      <c r="AZ4">
-        <v>0.2093023255813954</v>
-      </c>
-      <c r="BA4">
-        <v>0.2162790697674419</v>
-      </c>
-      <c r="BB4">
-        <v>0.2232558139534884</v>
-      </c>
-      <c r="BC4">
-        <v>0.2302325581395349</v>
-      </c>
-      <c r="BD4">
-        <v>0.2372093023255814</v>
-      </c>
-      <c r="BE4">
-        <v>0.2441860465116279</v>
-      </c>
-      <c r="BF4">
-        <v>0.2511627906976744</v>
-      </c>
-      <c r="BG4">
-        <v>0.2581395348837209</v>
-      </c>
-      <c r="BH4">
-        <v>0.2651162790697674</v>
-      </c>
-      <c r="BI4">
-        <v>0.2720930232558139</v>
-      </c>
-      <c r="BJ4">
-        <v>0.2790697674418605</v>
-      </c>
-      <c r="BK4">
-        <v>0.286046511627907</v>
-      </c>
-      <c r="BL4">
-        <v>0.2930232558139534</v>
-      </c>
       <c r="BM4">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="5" spans="1:65">
@@ -43398,133 +43398,133 @@
         <v>0</v>
       </c>
       <c r="W5">
-        <v>0.006976744186046512</v>
+        <v>0.01627906976744186</v>
       </c>
       <c r="X5">
-        <v>0.01395348837209302</v>
+        <v>0.03255813953488372</v>
       </c>
       <c r="Y5">
-        <v>0.02093023255813953</v>
+        <v>0.04883720930232558</v>
       </c>
       <c r="Z5">
-        <v>0.02790697674418605</v>
+        <v>0.06511627906976744</v>
       </c>
       <c r="AA5">
-        <v>0.03488372093023256</v>
+        <v>0.08139534883720929</v>
       </c>
       <c r="AB5">
-        <v>0.04186046511627907</v>
+        <v>0.09767441860465116</v>
       </c>
       <c r="AC5">
-        <v>0.04883720930232558</v>
+        <v>0.113953488372093</v>
       </c>
       <c r="AD5">
-        <v>0.05581395348837209</v>
+        <v>0.1302325581395349</v>
       </c>
       <c r="AE5">
-        <v>0.06279069767441861</v>
+        <v>0.1465116279069767</v>
       </c>
       <c r="AF5">
-        <v>0.06976744186046512</v>
+        <v>0.1627906976744186</v>
       </c>
       <c r="AG5">
-        <v>0.07674418604651163</v>
+        <v>0.1790697674418605</v>
       </c>
       <c r="AH5">
-        <v>0.08372093023255814</v>
+        <v>0.1953488372093023</v>
       </c>
       <c r="AI5">
-        <v>0.09069767441860464</v>
+        <v>0.2116279069767442</v>
       </c>
       <c r="AJ5">
-        <v>0.09767441860465116</v>
+        <v>0.2279069767441861</v>
       </c>
       <c r="AK5">
-        <v>0.1046511627906977</v>
+        <v>0.2441860465116279</v>
       </c>
       <c r="AL5">
-        <v>0.1116279069767442</v>
+        <v>0.2604651162790698</v>
       </c>
       <c r="AM5">
-        <v>0.1186046511627907</v>
+        <v>0.2767441860465116</v>
       </c>
       <c r="AN5">
-        <v>0.1255813953488372</v>
+        <v>0.2930232558139535</v>
       </c>
       <c r="AO5">
-        <v>0.1325581395348837</v>
+        <v>0.3093023255813953</v>
       </c>
       <c r="AP5">
-        <v>0.1395348837209302</v>
+        <v>0.3255813953488372</v>
       </c>
       <c r="AQ5">
-        <v>0.1465116279069767</v>
+        <v>0.341860465116279</v>
       </c>
       <c r="AR5">
-        <v>0.1534883720930233</v>
+        <v>0.3581395348837209</v>
       </c>
       <c r="AS5">
-        <v>0.1604651162790698</v>
+        <v>0.3744186046511627</v>
       </c>
       <c r="AT5">
-        <v>0.1674418604651163</v>
+        <v>0.3906976744186046</v>
       </c>
       <c r="AU5">
-        <v>0.1744186046511628</v>
+        <v>0.4069767441860465</v>
       </c>
       <c r="AV5">
-        <v>0.1813953488372093</v>
+        <v>0.4232558139534883</v>
       </c>
       <c r="AW5">
-        <v>0.1883720930232558</v>
+        <v>0.4395348837209302</v>
       </c>
       <c r="AX5">
-        <v>0.1953488372093023</v>
+        <v>0.4558139534883721</v>
       </c>
       <c r="AY5">
-        <v>0.2023255813953488</v>
+        <v>0.4720930232558139</v>
       </c>
       <c r="AZ5">
-        <v>0.2093023255813954</v>
+        <v>0.4883720930232558</v>
       </c>
       <c r="BA5">
-        <v>0.2162790697674419</v>
+        <v>0.5046511627906977</v>
       </c>
       <c r="BB5">
-        <v>0.2232558139534884</v>
+        <v>0.5209302325581395</v>
       </c>
       <c r="BC5">
-        <v>0.2302325581395349</v>
+        <v>0.5372093023255814</v>
       </c>
       <c r="BD5">
-        <v>0.2372093023255814</v>
+        <v>0.5534883720930232</v>
       </c>
       <c r="BE5">
-        <v>0.2441860465116279</v>
+        <v>0.5697674418604651</v>
       </c>
       <c r="BF5">
-        <v>0.2511627906976744</v>
+        <v>0.586046511627907</v>
       </c>
       <c r="BG5">
-        <v>0.2581395348837209</v>
+        <v>0.6023255813953488</v>
       </c>
       <c r="BH5">
-        <v>0.2651162790697674</v>
+        <v>0.6186046511627906</v>
       </c>
       <c r="BI5">
-        <v>0.2720930232558139</v>
+        <v>0.6348837209302325</v>
       </c>
       <c r="BJ5">
-        <v>0.2790697674418605</v>
+        <v>0.6511627906976744</v>
       </c>
       <c r="BK5">
-        <v>0.286046511627907</v>
+        <v>0.6674418604651162</v>
       </c>
       <c r="BL5">
-        <v>0.2930232558139534</v>
+        <v>0.6837209302325581</v>
       </c>
       <c r="BM5">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="6" spans="1:65">
@@ -43583,133 +43583,133 @@
         <v>0</v>
       </c>
       <c r="W6">
+        <v>0.002325581395348837</v>
+      </c>
+      <c r="X6">
         <v>0.004651162790697674</v>
       </c>
-      <c r="X6">
+      <c r="Y6">
+        <v>0.006976744186046512</v>
+      </c>
+      <c r="Z6">
         <v>0.009302325581395349</v>
       </c>
-      <c r="Y6">
+      <c r="AA6">
+        <v>0.01162790697674419</v>
+      </c>
+      <c r="AB6">
         <v>0.01395348837209302</v>
       </c>
-      <c r="Z6">
+      <c r="AC6">
+        <v>0.01627906976744186</v>
+      </c>
+      <c r="AD6">
         <v>0.0186046511627907</v>
       </c>
-      <c r="AA6">
+      <c r="AE6">
+        <v>0.02093023255813954</v>
+      </c>
+      <c r="AF6">
         <v>0.02325581395348837</v>
       </c>
-      <c r="AB6">
+      <c r="AG6">
+        <v>0.02558139534883721</v>
+      </c>
+      <c r="AH6">
         <v>0.02790697674418605</v>
       </c>
-      <c r="AC6">
+      <c r="AI6">
+        <v>0.03023255813953488</v>
+      </c>
+      <c r="AJ6">
         <v>0.03255813953488373</v>
       </c>
-      <c r="AD6">
+      <c r="AK6">
+        <v>0.03488372093023256</v>
+      </c>
+      <c r="AL6">
         <v>0.03720930232558139</v>
       </c>
-      <c r="AE6">
+      <c r="AM6">
+        <v>0.03953488372093023</v>
+      </c>
+      <c r="AN6">
         <v>0.04186046511627908</v>
       </c>
-      <c r="AF6">
+      <c r="AO6">
+        <v>0.04418604651162791</v>
+      </c>
+      <c r="AP6">
         <v>0.04651162790697674</v>
       </c>
-      <c r="AG6">
+      <c r="AQ6">
+        <v>0.04883720930232558</v>
+      </c>
+      <c r="AR6">
         <v>0.05116279069767442</v>
       </c>
-      <c r="AH6">
+      <c r="AS6">
+        <v>0.05348837209302326</v>
+      </c>
+      <c r="AT6">
         <v>0.05581395348837209</v>
       </c>
-      <c r="AI6">
+      <c r="AU6">
+        <v>0.05813953488372094</v>
+      </c>
+      <c r="AV6">
         <v>0.06046511627906977</v>
       </c>
-      <c r="AJ6">
+      <c r="AW6">
+        <v>0.06279069767441861</v>
+      </c>
+      <c r="AX6">
         <v>0.06511627906976745</v>
       </c>
-      <c r="AK6">
+      <c r="AY6">
+        <v>0.06744186046511629</v>
+      </c>
+      <c r="AZ6">
         <v>0.06976744186046512</v>
       </c>
-      <c r="AL6">
+      <c r="BA6">
+        <v>0.07209302325581395</v>
+      </c>
+      <c r="BB6">
         <v>0.07441860465116279</v>
       </c>
-      <c r="AM6">
+      <c r="BC6">
+        <v>0.07674418604651163</v>
+      </c>
+      <c r="BD6">
         <v>0.07906976744186046</v>
       </c>
-      <c r="AN6">
+      <c r="BE6">
+        <v>0.08139534883720931</v>
+      </c>
+      <c r="BF6">
         <v>0.08372093023255815</v>
       </c>
-      <c r="AO6">
+      <c r="BG6">
+        <v>0.08604651162790698</v>
+      </c>
+      <c r="BH6">
         <v>0.08837209302325583</v>
       </c>
-      <c r="AP6">
+      <c r="BI6">
+        <v>0.09069767441860466</v>
+      </c>
+      <c r="BJ6">
         <v>0.09302325581395349</v>
       </c>
-      <c r="AQ6">
+      <c r="BK6">
+        <v>0.09534883720930233</v>
+      </c>
+      <c r="BL6">
         <v>0.09767441860465116</v>
       </c>
-      <c r="AR6">
-        <v>0.1023255813953488</v>
-      </c>
-      <c r="AS6">
-        <v>0.1069767441860465</v>
-      </c>
-      <c r="AT6">
-        <v>0.1116279069767442</v>
-      </c>
-      <c r="AU6">
-        <v>0.1162790697674419</v>
-      </c>
-      <c r="AV6">
-        <v>0.1209302325581395</v>
-      </c>
-      <c r="AW6">
-        <v>0.1255813953488372</v>
-      </c>
-      <c r="AX6">
-        <v>0.1302325581395349</v>
-      </c>
-      <c r="AY6">
-        <v>0.1348837209302326</v>
-      </c>
-      <c r="AZ6">
-        <v>0.1395348837209302</v>
-      </c>
-      <c r="BA6">
-        <v>0.1441860465116279</v>
-      </c>
-      <c r="BB6">
-        <v>0.1488372093023256</v>
-      </c>
-      <c r="BC6">
-        <v>0.1534883720930233</v>
-      </c>
-      <c r="BD6">
-        <v>0.1581395348837209</v>
-      </c>
-      <c r="BE6">
-        <v>0.1627906976744186</v>
-      </c>
-      <c r="BF6">
-        <v>0.1674418604651163</v>
-      </c>
-      <c r="BG6">
-        <v>0.172093023255814</v>
-      </c>
-      <c r="BH6">
-        <v>0.1767441860465117</v>
-      </c>
-      <c r="BI6">
-        <v>0.1813953488372093</v>
-      </c>
-      <c r="BJ6">
-        <v>0.186046511627907</v>
-      </c>
-      <c r="BK6">
-        <v>0.1906976744186047</v>
-      </c>
-      <c r="BL6">
-        <v>0.1953488372093023</v>
-      </c>
       <c r="BM6">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="7" spans="1:65">
@@ -43768,133 +43768,133 @@
         <v>0</v>
       </c>
       <c r="W7">
+        <v>0.002325581395348837</v>
+      </c>
+      <c r="X7">
         <v>0.004651162790697674</v>
       </c>
-      <c r="X7">
+      <c r="Y7">
+        <v>0.006976744186046512</v>
+      </c>
+      <c r="Z7">
         <v>0.009302325581395349</v>
       </c>
-      <c r="Y7">
+      <c r="AA7">
+        <v>0.01162790697674419</v>
+      </c>
+      <c r="AB7">
         <v>0.01395348837209302</v>
       </c>
-      <c r="Z7">
+      <c r="AC7">
+        <v>0.01627906976744186</v>
+      </c>
+      <c r="AD7">
         <v>0.0186046511627907</v>
       </c>
-      <c r="AA7">
+      <c r="AE7">
+        <v>0.02093023255813954</v>
+      </c>
+      <c r="AF7">
         <v>0.02325581395348837</v>
       </c>
-      <c r="AB7">
+      <c r="AG7">
+        <v>0.02558139534883721</v>
+      </c>
+      <c r="AH7">
         <v>0.02790697674418605</v>
       </c>
-      <c r="AC7">
+      <c r="AI7">
+        <v>0.03023255813953488</v>
+      </c>
+      <c r="AJ7">
         <v>0.03255813953488373</v>
       </c>
-      <c r="AD7">
+      <c r="AK7">
+        <v>0.03488372093023256</v>
+      </c>
+      <c r="AL7">
         <v>0.03720930232558139</v>
       </c>
-      <c r="AE7">
+      <c r="AM7">
+        <v>0.03953488372093023</v>
+      </c>
+      <c r="AN7">
         <v>0.04186046511627908</v>
       </c>
-      <c r="AF7">
+      <c r="AO7">
+        <v>0.04418604651162791</v>
+      </c>
+      <c r="AP7">
         <v>0.04651162790697674</v>
       </c>
-      <c r="AG7">
+      <c r="AQ7">
+        <v>0.04883720930232558</v>
+      </c>
+      <c r="AR7">
         <v>0.05116279069767442</v>
       </c>
-      <c r="AH7">
+      <c r="AS7">
+        <v>0.05348837209302326</v>
+      </c>
+      <c r="AT7">
         <v>0.05581395348837209</v>
       </c>
-      <c r="AI7">
+      <c r="AU7">
+        <v>0.05813953488372094</v>
+      </c>
+      <c r="AV7">
         <v>0.06046511627906977</v>
       </c>
-      <c r="AJ7">
+      <c r="AW7">
+        <v>0.06279069767441861</v>
+      </c>
+      <c r="AX7">
         <v>0.06511627906976745</v>
       </c>
-      <c r="AK7">
+      <c r="AY7">
+        <v>0.06744186046511629</v>
+      </c>
+      <c r="AZ7">
         <v>0.06976744186046512</v>
       </c>
-      <c r="AL7">
+      <c r="BA7">
+        <v>0.07209302325581395</v>
+      </c>
+      <c r="BB7">
         <v>0.07441860465116279</v>
       </c>
-      <c r="AM7">
+      <c r="BC7">
+        <v>0.07674418604651163</v>
+      </c>
+      <c r="BD7">
         <v>0.07906976744186046</v>
       </c>
-      <c r="AN7">
+      <c r="BE7">
+        <v>0.08139534883720931</v>
+      </c>
+      <c r="BF7">
         <v>0.08372093023255815</v>
       </c>
-      <c r="AO7">
+      <c r="BG7">
+        <v>0.08604651162790698</v>
+      </c>
+      <c r="BH7">
         <v>0.08837209302325583</v>
       </c>
-      <c r="AP7">
+      <c r="BI7">
+        <v>0.09069767441860466</v>
+      </c>
+      <c r="BJ7">
         <v>0.09302325581395349</v>
       </c>
-      <c r="AQ7">
+      <c r="BK7">
+        <v>0.09534883720930233</v>
+      </c>
+      <c r="BL7">
         <v>0.09767441860465116</v>
       </c>
-      <c r="AR7">
-        <v>0.1023255813953488</v>
-      </c>
-      <c r="AS7">
-        <v>0.1069767441860465</v>
-      </c>
-      <c r="AT7">
-        <v>0.1116279069767442</v>
-      </c>
-      <c r="AU7">
-        <v>0.1162790697674419</v>
-      </c>
-      <c r="AV7">
-        <v>0.1209302325581395</v>
-      </c>
-      <c r="AW7">
-        <v>0.1255813953488372</v>
-      </c>
-      <c r="AX7">
-        <v>0.1302325581395349</v>
-      </c>
-      <c r="AY7">
-        <v>0.1348837209302326</v>
-      </c>
-      <c r="AZ7">
-        <v>0.1395348837209302</v>
-      </c>
-      <c r="BA7">
-        <v>0.1441860465116279</v>
-      </c>
-      <c r="BB7">
-        <v>0.1488372093023256</v>
-      </c>
-      <c r="BC7">
-        <v>0.1534883720930233</v>
-      </c>
-      <c r="BD7">
-        <v>0.1581395348837209</v>
-      </c>
-      <c r="BE7">
-        <v>0.1627906976744186</v>
-      </c>
-      <c r="BF7">
-        <v>0.1674418604651163</v>
-      </c>
-      <c r="BG7">
-        <v>0.172093023255814</v>
-      </c>
-      <c r="BH7">
-        <v>0.1767441860465117</v>
-      </c>
-      <c r="BI7">
-        <v>0.1813953488372093</v>
-      </c>
-      <c r="BJ7">
-        <v>0.186046511627907</v>
-      </c>
-      <c r="BK7">
-        <v>0.1906976744186047</v>
-      </c>
-      <c r="BL7">
-        <v>0.1953488372093023</v>
-      </c>
       <c r="BM7">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="8" spans="1:65">
@@ -44031,31 +44031,31 @@
         <v>0.3953488372093024</v>
       </c>
       <c r="AW8">
-        <v>0.3720930232558139</v>
+        <v>0.372093023255814</v>
       </c>
       <c r="AX8">
-        <v>0.3488372093023255</v>
+        <v>0.3488372093023256</v>
       </c>
       <c r="AY8">
-        <v>0.3255813953488372</v>
+        <v>0.3255813953488373</v>
       </c>
       <c r="AZ8">
-        <v>0.3023255813953488</v>
+        <v>0.3023255813953489</v>
       </c>
       <c r="BA8">
-        <v>0.2790697674418605</v>
+        <v>0.2790697674418606</v>
       </c>
       <c r="BB8">
-        <v>0.2558139534883721</v>
+        <v>0.2558139534883722</v>
       </c>
       <c r="BC8">
-        <v>0.2325581395348837</v>
+        <v>0.2325581395348838</v>
       </c>
       <c r="BD8">
-        <v>0.2093023255813954</v>
+        <v>0.2093023255813955</v>
       </c>
       <c r="BE8">
-        <v>0.186046511627907</v>
+        <v>0.1860465116279071</v>
       </c>
       <c r="BF8">
         <v>0.1627906976744186</v>
@@ -44064,22 +44064,22 @@
         <v>0.1395348837209303</v>
       </c>
       <c r="BH8">
-        <v>0.1162790697674418</v>
+        <v>0.1162790697674419</v>
       </c>
       <c r="BI8">
-        <v>0.09302325581395354</v>
+        <v>0.09302325581395364</v>
       </c>
       <c r="BJ8">
-        <v>0.06976744186046513</v>
+        <v>0.06976744186046523</v>
       </c>
       <c r="BK8">
-        <v>0.04651162790697672</v>
+        <v>0.04651162790697682</v>
       </c>
       <c r="BL8">
-        <v>0.02325581395348841</v>
+        <v>0.02325581395348852</v>
       </c>
       <c r="BM8">
-        <v>0</v>
+        <v>1.110223024625157E-16</v>
       </c>
     </row>
     <row r="9" spans="1:65">
@@ -46331,133 +46331,133 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="W21">
-        <v>0.09162790697674419</v>
+        <v>0.09046511627906978</v>
       </c>
       <c r="X21">
-        <v>0.1132558139534884</v>
+        <v>0.1109302325581396</v>
       </c>
       <c r="Y21">
-        <v>0.1348837209302325</v>
+        <v>0.1313953488372093</v>
       </c>
       <c r="Z21">
-        <v>0.1565116279069768</v>
+        <v>0.1518604651162791</v>
       </c>
       <c r="AA21">
-        <v>0.1781395348837209</v>
+        <v>0.1723255813953488</v>
       </c>
       <c r="AB21">
-        <v>0.1997674418604651</v>
+        <v>0.1927906976744186</v>
       </c>
       <c r="AC21">
-        <v>0.2213953488372093</v>
+        <v>0.2132558139534884</v>
       </c>
       <c r="AD21">
-        <v>0.2430232558139535</v>
+        <v>0.2337209302325581</v>
       </c>
       <c r="AE21">
-        <v>0.2646511627906977</v>
+        <v>0.2541860465116279</v>
       </c>
       <c r="AF21">
-        <v>0.2862790697674419</v>
+        <v>0.2746511627906977</v>
       </c>
       <c r="AG21">
-        <v>0.307906976744186</v>
+        <v>0.2951162790697675</v>
       </c>
       <c r="AH21">
-        <v>0.3295348837209302</v>
+        <v>0.3155813953488372</v>
       </c>
       <c r="AI21">
-        <v>0.3511627906976744</v>
+        <v>0.3360465116279069</v>
       </c>
       <c r="AJ21">
-        <v>0.3727906976744186</v>
+        <v>0.3565116279069768</v>
       </c>
       <c r="AK21">
-        <v>0.3944186046511628</v>
+        <v>0.3769767441860465</v>
       </c>
       <c r="AL21">
-        <v>0.416046511627907</v>
+        <v>0.3974418604651163</v>
       </c>
       <c r="AM21">
-        <v>0.4376744186046512</v>
+        <v>0.417906976744186</v>
       </c>
       <c r="AN21">
-        <v>0.4593023255813954</v>
+        <v>0.4383720930232559</v>
       </c>
       <c r="AO21">
-        <v>0.4809302325581395</v>
+        <v>0.4588372093023256</v>
       </c>
       <c r="AP21">
-        <v>0.5025581395348837</v>
+        <v>0.4793023255813953</v>
       </c>
       <c r="AQ21">
-        <v>0.5241860465116279</v>
+        <v>0.4997674418604651</v>
       </c>
       <c r="AR21">
-        <v>0.5458139534883721</v>
+        <v>0.5202325581395348</v>
       </c>
       <c r="AS21">
-        <v>0.5674418604651162</v>
+        <v>0.5406976744186046</v>
       </c>
       <c r="AT21">
-        <v>0.5890697674418605</v>
+        <v>0.5611627906976744</v>
       </c>
       <c r="AU21">
-        <v>0.6106976744186047</v>
+        <v>0.5816279069767442</v>
       </c>
       <c r="AV21">
-        <v>0.6323255813953488</v>
+        <v>0.6020930232558138</v>
       </c>
       <c r="AW21">
-        <v>0.653953488372093</v>
+        <v>0.6225581395348837</v>
       </c>
       <c r="AX21">
-        <v>0.6755813953488372</v>
+        <v>0.6430232558139535</v>
       </c>
       <c r="AY21">
-        <v>0.6972093023255814</v>
+        <v>0.6634883720930232</v>
       </c>
       <c r="AZ21">
-        <v>0.7188372093023256</v>
+        <v>0.683953488372093</v>
       </c>
       <c r="BA21">
-        <v>0.7404651162790697</v>
+        <v>0.7044186046511628</v>
       </c>
       <c r="BB21">
-        <v>0.762093023255814</v>
+        <v>0.7248837209302326</v>
       </c>
       <c r="BC21">
-        <v>0.7837209302325582</v>
+        <v>0.7453488372093023</v>
       </c>
       <c r="BD21">
-        <v>0.8053488372093023</v>
+        <v>0.765813953488372</v>
       </c>
       <c r="BE21">
-        <v>0.8269767441860465</v>
+        <v>0.7862790697674418</v>
       </c>
       <c r="BF21">
-        <v>0.8486046511627907</v>
+        <v>0.8067441860465117</v>
       </c>
       <c r="BG21">
-        <v>0.8702325581395348</v>
+        <v>0.8272093023255813</v>
       </c>
       <c r="BH21">
-        <v>0.891860465116279</v>
+        <v>0.8476744186046511</v>
       </c>
       <c r="BI21">
-        <v>0.9134883720930232</v>
+        <v>0.8681395348837209</v>
       </c>
       <c r="BJ21">
-        <v>0.9351162790697675</v>
+        <v>0.8886046511627906</v>
       </c>
       <c r="BK21">
-        <v>0.9567441860465117</v>
+        <v>0.9090697674418605</v>
       </c>
       <c r="BL21">
-        <v>0.9783720930232558</v>
+        <v>0.9295348837209302</v>
       </c>
       <c r="BM21">
-        <v>1</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="22" spans="1:65">
@@ -46513,133 +46513,133 @@
         <v>0.5</v>
       </c>
       <c r="W22">
-        <v>0.5116279069767442</v>
+        <v>0.5104651162790698</v>
       </c>
       <c r="X22">
-        <v>0.5232558139534884</v>
+        <v>0.5209302325581395</v>
       </c>
       <c r="Y22">
-        <v>0.5348837209302325</v>
+        <v>0.5313953488372093</v>
       </c>
       <c r="Z22">
-        <v>0.5465116279069768</v>
+        <v>0.5418604651162791</v>
       </c>
       <c r="AA22">
-        <v>0.5581395348837209</v>
+        <v>0.5523255813953488</v>
       </c>
       <c r="AB22">
-        <v>0.5697674418604651</v>
+        <v>0.5627906976744186</v>
       </c>
       <c r="AC22">
-        <v>0.5813953488372092</v>
+        <v>0.5732558139534883</v>
       </c>
       <c r="AD22">
-        <v>0.5930232558139534</v>
+        <v>0.5837209302325581</v>
       </c>
       <c r="AE22">
+        <v>0.5941860465116279</v>
+      </c>
+      <c r="AF22">
         <v>0.6046511627906976</v>
       </c>
-      <c r="AF22">
-        <v>0.6162790697674418</v>
-      </c>
       <c r="AG22">
-        <v>0.6279069767441861</v>
+        <v>0.6151162790697674</v>
       </c>
       <c r="AH22">
-        <v>0.6395348837209303</v>
+        <v>0.6255813953488372</v>
       </c>
       <c r="AI22">
-        <v>0.6511627906976745</v>
+        <v>0.6360465116279069</v>
       </c>
       <c r="AJ22">
-        <v>0.6627906976744187</v>
+        <v>0.6465116279069767</v>
       </c>
       <c r="AK22">
-        <v>0.6744186046511629</v>
+        <v>0.6569767441860466</v>
       </c>
       <c r="AL22">
-        <v>0.686046511627907</v>
+        <v>0.6674418604651162</v>
       </c>
       <c r="AM22">
-        <v>0.6976744186046511</v>
+        <v>0.677906976744186</v>
       </c>
       <c r="AN22">
+        <v>0.6883720930232557</v>
+      </c>
+      <c r="AO22">
+        <v>0.6988372093023256</v>
+      </c>
+      <c r="AP22">
         <v>0.7093023255813953</v>
       </c>
-      <c r="AO22">
-        <v>0.7209302325581395</v>
-      </c>
-      <c r="AP22">
-        <v>0.7325581395348837</v>
-      </c>
       <c r="AQ22">
-        <v>0.7441860465116279</v>
+        <v>0.7197674418604652</v>
       </c>
       <c r="AR22">
-        <v>0.7558139534883721</v>
+        <v>0.7302325581395348</v>
       </c>
       <c r="AS22">
-        <v>0.7674418604651163</v>
+        <v>0.7406976744186047</v>
       </c>
       <c r="AT22">
-        <v>0.7790697674418605</v>
+        <v>0.7511627906976743</v>
       </c>
       <c r="AU22">
-        <v>0.7906976744186047</v>
+        <v>0.7616279069767442</v>
       </c>
       <c r="AV22">
-        <v>0.8023255813953488</v>
+        <v>0.7720930232558139</v>
       </c>
       <c r="AW22">
-        <v>0.813953488372093</v>
+        <v>0.7825581395348837</v>
       </c>
       <c r="AX22">
-        <v>0.8255813953488372</v>
+        <v>0.7930232558139535</v>
       </c>
       <c r="AY22">
-        <v>0.8372093023255813</v>
+        <v>0.8034883720930233</v>
       </c>
       <c r="AZ22">
-        <v>0.8488372093023255</v>
+        <v>0.8139534883720929</v>
       </c>
       <c r="BA22">
-        <v>0.8604651162790697</v>
+        <v>0.8244186046511628</v>
       </c>
       <c r="BB22">
-        <v>0.8720930232558139</v>
+        <v>0.8348837209302326</v>
       </c>
       <c r="BC22">
-        <v>0.8837209302325582</v>
+        <v>0.8453488372093023</v>
       </c>
       <c r="BD22">
-        <v>0.8953488372093024</v>
+        <v>0.855813953488372</v>
       </c>
       <c r="BE22">
-        <v>0.9069767441860466</v>
+        <v>0.8662790697674418</v>
       </c>
       <c r="BF22">
-        <v>0.9186046511627908</v>
+        <v>0.8767441860465117</v>
       </c>
       <c r="BG22">
-        <v>0.9302325581395349</v>
+        <v>0.8872093023255814</v>
       </c>
       <c r="BH22">
-        <v>0.9418604651162791</v>
+        <v>0.8976744186046511</v>
       </c>
       <c r="BI22">
-        <v>0.9534883720930232</v>
+        <v>0.9081395348837209</v>
       </c>
       <c r="BJ22">
-        <v>0.9651162790697674</v>
+        <v>0.9186046511627906</v>
       </c>
       <c r="BK22">
-        <v>0.9767441860465116</v>
+        <v>0.9290697674418604</v>
       </c>
       <c r="BL22">
-        <v>0.9883720930232558</v>
+        <v>0.9395348837209302</v>
       </c>
       <c r="BM22">
-        <v>1</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="23" spans="1:65">
@@ -48521,133 +48521,133 @@
         <v>0.95</v>
       </c>
       <c r="W33">
-        <v>0.9511627906976744</v>
+        <v>0.95</v>
       </c>
       <c r="X33">
-        <v>0.9523255813953488</v>
+        <v>0.9500000000000001</v>
       </c>
       <c r="Y33">
-        <v>0.9534883720930232</v>
+        <v>0.95</v>
       </c>
       <c r="Z33">
-        <v>0.9546511627906977</v>
+        <v>0.95</v>
       </c>
       <c r="AA33">
-        <v>0.9558139534883721</v>
+        <v>0.95</v>
       </c>
       <c r="AB33">
-        <v>0.9569767441860465</v>
+        <v>0.95</v>
       </c>
       <c r="AC33">
-        <v>0.9581395348837209</v>
+        <v>0.95</v>
       </c>
       <c r="AD33">
-        <v>0.9593023255813953</v>
+        <v>0.95</v>
       </c>
       <c r="AE33">
-        <v>0.9604651162790697</v>
+        <v>0.95</v>
       </c>
       <c r="AF33">
-        <v>0.9616279069767442</v>
+        <v>0.95</v>
       </c>
       <c r="AG33">
-        <v>0.9627906976744186</v>
+        <v>0.95</v>
       </c>
       <c r="AH33">
-        <v>0.963953488372093</v>
+        <v>0.95</v>
       </c>
       <c r="AI33">
-        <v>0.9651162790697674</v>
+        <v>0.95</v>
       </c>
       <c r="AJ33">
-        <v>0.9662790697674418</v>
+        <v>0.95</v>
       </c>
       <c r="AK33">
-        <v>0.9674418604651163</v>
+        <v>0.95</v>
       </c>
       <c r="AL33">
-        <v>0.9686046511627907</v>
+        <v>0.95</v>
       </c>
       <c r="AM33">
-        <v>0.9697674418604649</v>
+        <v>0.9499999999999998</v>
       </c>
       <c r="AN33">
-        <v>0.9709302325581395</v>
+        <v>0.95</v>
       </c>
       <c r="AO33">
-        <v>0.9720930232558139</v>
+        <v>0.95</v>
       </c>
       <c r="AP33">
-        <v>0.9732558139534884</v>
+        <v>0.95</v>
       </c>
       <c r="AQ33">
-        <v>0.9744186046511627</v>
+        <v>0.95</v>
       </c>
       <c r="AR33">
-        <v>0.9755813953488373</v>
+        <v>0.95</v>
       </c>
       <c r="AS33">
-        <v>0.9767441860465116</v>
+        <v>0.95</v>
       </c>
       <c r="AT33">
-        <v>0.977906976744186</v>
+        <v>0.95</v>
       </c>
       <c r="AU33">
-        <v>0.9790697674418605</v>
+        <v>0.95</v>
       </c>
       <c r="AV33">
-        <v>0.9802325581395348</v>
+        <v>0.95</v>
       </c>
       <c r="AW33">
-        <v>0.9813953488372094</v>
+        <v>0.95</v>
       </c>
       <c r="AX33">
-        <v>0.9825581395348837</v>
+        <v>0.95</v>
       </c>
       <c r="AY33">
-        <v>0.9837209302325581</v>
+        <v>0.95</v>
       </c>
       <c r="AZ33">
-        <v>0.9848837209302326</v>
+        <v>0.95</v>
       </c>
       <c r="BA33">
-        <v>0.9860465116279069</v>
+        <v>0.95</v>
       </c>
       <c r="BB33">
-        <v>0.9872093023255814</v>
+        <v>0.95</v>
       </c>
       <c r="BC33">
-        <v>0.9883720930232558</v>
+        <v>0.95</v>
       </c>
       <c r="BD33">
-        <v>0.9895348837209302</v>
+        <v>0.95</v>
       </c>
       <c r="BE33">
-        <v>0.9906976744186047</v>
+        <v>0.95</v>
       </c>
       <c r="BF33">
-        <v>0.991860465116279</v>
+        <v>0.95</v>
       </c>
       <c r="BG33">
-        <v>0.9930232558139535</v>
+        <v>0.95</v>
       </c>
       <c r="BH33">
-        <v>0.9941860465116279</v>
+        <v>0.95</v>
       </c>
       <c r="BI33">
-        <v>0.9953488372093023</v>
+        <v>0.95</v>
       </c>
       <c r="BJ33">
-        <v>0.9965116279069768</v>
+        <v>0.95</v>
       </c>
       <c r="BK33">
-        <v>0.9976744186046511</v>
+        <v>0.95</v>
       </c>
       <c r="BL33">
-        <v>0.9988372093023256</v>
+        <v>0.95</v>
       </c>
       <c r="BM33">
-        <v>1</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="34" spans="1:65">

</xml_diff>